<commit_message>
Daily NSE scan: 2026-10-16
</commit_message>
<xml_diff>
--- a/output/2026-10-16/enriched_analysis.xlsx
+++ b/output/2026-10-16/enriched_analysis.xlsx
@@ -1396,7 +1396,7 @@
         <v>0.021</v>
       </c>
       <c r="W4" t="n">
-        <v>3434</v>
+        <v>3436</v>
       </c>
       <c r="X4" t="n">
         <v>15.6</v>
@@ -1628,7 +1628,7 @@
         <v>0.045</v>
       </c>
       <c r="W5" t="n">
-        <v>2927</v>
+        <v>2928</v>
       </c>
       <c r="X5" t="n">
         <v>10.1</v>
@@ -1857,13 +1857,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1.041</v>
+        <v>1.044</v>
       </c>
       <c r="W6" t="n">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="X6" t="n">
-        <v>86.90000000000001</v>
+        <v>86.5</v>
       </c>
       <c r="Y6" t="n">
         <v>111</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.103</v>
+        <v>1.14</v>
       </c>
       <c r="W7" t="n">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="X7" t="n">
-        <v>7.73</v>
+        <v>7.47</v>
       </c>
       <c r="Y7" t="n">
         <v>17</v>
@@ -2324,7 +2324,7 @@
         <v>0.048</v>
       </c>
       <c r="W8" t="n">
-        <v>14877</v>
+        <v>14891</v>
       </c>
       <c r="X8" t="n">
         <v>37.9</v>
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>2.299</v>
+        <v>2.315</v>
       </c>
       <c r="W9" t="n">
-        <v>2553</v>
+        <v>2535</v>
       </c>
       <c r="X9" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Y9" t="n">
         <v>6</v>
@@ -2788,7 +2788,7 @@
         <v>0.052</v>
       </c>
       <c r="W10" t="n">
-        <v>1573</v>
+        <v>1572</v>
       </c>
       <c r="X10" t="n">
         <v>21.2</v>
@@ -3249,10 +3249,10 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.47</v>
+        <v>0.469</v>
       </c>
       <c r="W12" t="n">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="X12" t="n">
         <v>15.4</v>
@@ -3481,13 +3481,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.123</v>
+        <v>0.126</v>
       </c>
       <c r="W13" t="n">
-        <v>706</v>
+        <v>689</v>
       </c>
       <c r="X13" t="n">
-        <v>26.6</v>
+        <v>26</v>
       </c>
       <c r="Y13" t="n">
         <v>13</v>
@@ -3716,10 +3716,10 @@
         <v>0.127</v>
       </c>
       <c r="W14" t="n">
-        <v>2477</v>
+        <v>2469</v>
       </c>
       <c r="X14" t="n">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="Y14" t="n">
         <v>-3</v>
@@ -3948,10 +3948,10 @@
         <v>0.064</v>
       </c>
       <c r="W15" t="n">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="X15" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="Y15" t="n">
         <v>19</v>
@@ -4408,7 +4408,7 @@
         <v>0.178</v>
       </c>
       <c r="W17" t="n">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="X17" t="n">
         <v>39.3</v>
@@ -4640,10 +4640,10 @@
         <v>0.057</v>
       </c>
       <c r="W18" t="n">
-        <v>2236</v>
+        <v>2225</v>
       </c>
       <c r="X18" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Y18" t="n">
         <v>13</v>
@@ -4869,13 +4869,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>1.239</v>
+        <v>1.231</v>
       </c>
       <c r="W19" t="n">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="X19" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Y19" t="n">
         <v>22</v>
@@ -5104,10 +5104,10 @@
         <v>0.241</v>
       </c>
       <c r="W20" t="n">
-        <v>1429</v>
+        <v>1426</v>
       </c>
       <c r="X20" t="n">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="Y20" t="n">
         <v>8</v>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.161</v>
+        <v>0.162</v>
       </c>
       <c r="W21" t="n">
-        <v>688</v>
+        <v>682</v>
       </c>
       <c r="X21" t="n">
-        <v>57.5</v>
+        <v>57</v>
       </c>
       <c r="Y21" t="n">
         <v>3</v>
@@ -5563,13 +5563,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>1.509</v>
+        <v>1.513</v>
       </c>
       <c r="W22" t="n">
-        <v>8970</v>
+        <v>8944</v>
       </c>
       <c r="X22" t="n">
-        <v>1510</v>
+        <v>1506</v>
       </c>
       <c r="Y22" t="n">
         <v>-53</v>
@@ -5795,10 +5795,10 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>1.785</v>
+        <v>1.799</v>
       </c>
       <c r="W23" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="n">
@@ -6028,10 +6028,10 @@
         <v>0.068</v>
       </c>
       <c r="W24" t="n">
-        <v>1641</v>
+        <v>1639</v>
       </c>
       <c r="X24" t="n">
-        <v>37.7</v>
+        <v>37.6</v>
       </c>
       <c r="Y24" t="n">
         <v>20</v>
@@ -6257,10 +6257,10 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>3.169</v>
+        <v>3.179</v>
       </c>
       <c r="W25" t="n">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="X25" t="n">
         <v>18.7</v>
@@ -6483,13 +6483,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.577</v>
+        <v>0.579</v>
       </c>
       <c r="W26" t="n">
-        <v>2474</v>
+        <v>2468</v>
       </c>
       <c r="X26" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="Y26" t="n">
         <v>8</v>
@@ -6718,7 +6718,7 @@
         <v>0.103</v>
       </c>
       <c r="W27" t="n">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="X27" t="n">
         <v>36.3</v>
@@ -6941,13 +6941,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.319</v>
+        <v>0.318</v>
       </c>
       <c r="W28" t="n">
-        <v>59591</v>
+        <v>59742</v>
       </c>
       <c r="X28" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="Y28" t="n">
         <v>5</v>
@@ -7173,13 +7173,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.548</v>
+        <v>0.549</v>
       </c>
       <c r="W29" t="n">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="X29" t="n">
-        <v>16</v>
+        <v>15.9</v>
       </c>
       <c r="Y29" t="n">
         <v>13</v>
@@ -7405,13 +7405,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.339</v>
+        <v>0.341</v>
       </c>
       <c r="W30" t="n">
-        <v>954</v>
+        <v>948</v>
       </c>
       <c r="X30" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="Y30" t="n">
         <v>13</v>
@@ -7640,7 +7640,7 @@
         <v>0.148</v>
       </c>
       <c r="W31" t="n">
-        <v>1423</v>
+        <v>1426</v>
       </c>
       <c r="X31" t="n">
         <v>14.2</v>
@@ -8101,13 +8101,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.093</v>
+        <v>0.091</v>
       </c>
       <c r="W33" t="n">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="X33" t="n">
-        <v>9.98</v>
+        <v>10.2</v>
       </c>
       <c r="Y33" t="n">
         <v>-5</v>
@@ -8336,10 +8336,10 @@
         <v>0.121</v>
       </c>
       <c r="W34" t="n">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="X34" t="n">
-        <v>14.6</v>
+        <v>14.5</v>
       </c>
       <c r="Y34" t="n">
         <v>-1</v>
@@ -8565,13 +8565,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>1.671</v>
+        <v>1.633</v>
       </c>
       <c r="W35" t="n">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="X35" t="n">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="Y35" t="n">
         <v>-14</v>
@@ -8803,7 +8803,7 @@
         <v>176</v>
       </c>
       <c r="X36" t="n">
-        <v>5.14</v>
+        <v>5.16</v>
       </c>
       <c r="Y36" t="n">
         <v>31</v>
@@ -9025,13 +9025,13 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>1.136</v>
+        <v>1.135</v>
       </c>
       <c r="W37" t="n">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="X37" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Y37" t="n">
         <v>12</v>
@@ -9260,10 +9260,10 @@
         <v>0.174</v>
       </c>
       <c r="W38" t="n">
-        <v>3678</v>
+        <v>3669</v>
       </c>
       <c r="X38" t="n">
-        <v>6.93</v>
+        <v>6.91</v>
       </c>
       <c r="Y38" t="n">
         <v>2</v>
@@ -9455,7 +9455,7 @@
         <v>-4</v>
       </c>
       <c r="L39" t="n">
-        <v>75</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="M39" t="n">
         <v>4.84</v>
@@ -9492,7 +9492,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W39" t="n">
-        <v>54802</v>
+        <v>54808</v>
       </c>
       <c r="X39" t="n">
         <v>46.4</v>
@@ -9724,7 +9724,7 @@
         <v>0.01</v>
       </c>
       <c r="W40" t="n">
-        <v>15211</v>
+        <v>15205</v>
       </c>
       <c r="X40" t="n">
         <v>14</v>
@@ -9955,7 +9955,7 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="n">
-        <v>5.96</v>
+        <v>5.97</v>
       </c>
       <c r="Y41" t="n">
         <v>-68</v>
@@ -10184,7 +10184,7 @@
         <v>0.004</v>
       </c>
       <c r="W42" t="n">
-        <v>45053</v>
+        <v>45157</v>
       </c>
       <c r="X42" t="n">
         <v>334</v>
@@ -10413,13 +10413,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.372</v>
+        <v>0.374</v>
       </c>
       <c r="W43" t="n">
-        <v>1059</v>
+        <v>1052</v>
       </c>
       <c r="X43" t="n">
-        <v>53.9</v>
+        <v>53.6</v>
       </c>
       <c r="Y43" t="n">
         <v>21</v>
@@ -10645,13 +10645,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.529</v>
+        <v>0.525</v>
       </c>
       <c r="W44" t="n">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="X44" t="n">
-        <v>35</v>
+        <v>35.2</v>
       </c>
       <c r="Y44" t="n">
         <v>21</v>
@@ -10880,7 +10880,7 @@
         <v>0.045</v>
       </c>
       <c r="W45" t="n">
-        <v>5170</v>
+        <v>5172</v>
       </c>
       <c r="X45" t="n">
         <v>26.9</v>
@@ -11344,10 +11344,10 @@
         <v>0.043</v>
       </c>
       <c r="W47" t="n">
-        <v>1607</v>
+        <v>1614</v>
       </c>
       <c r="X47" t="n">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="Y47" t="n">
         <v>10</v>
@@ -11579,7 +11579,7 @@
         <v>210</v>
       </c>
       <c r="X48" t="n">
-        <v>36.4</v>
+        <v>36.3</v>
       </c>
       <c r="Y48" t="n">
         <v>-44</v>
@@ -11808,10 +11808,10 @@
         <v>0.272</v>
       </c>
       <c r="W49" t="n">
-        <v>955</v>
+        <v>958</v>
       </c>
       <c r="X49" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="Y49" t="n">
         <v>9</v>
@@ -12037,10 +12037,10 @@
         </is>
       </c>
       <c r="V50" t="n">
-        <v>4.583</v>
+        <v>4.601</v>
       </c>
       <c r="W50" t="n">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="X50" t="inlineStr"/>
       <c r="Y50" t="n">
@@ -12273,7 +12273,7 @@
         <v>349</v>
       </c>
       <c r="X51" t="n">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="Y51" t="n">
         <v>-61</v>
@@ -12721,13 +12721,13 @@
         </is>
       </c>
       <c r="V53" t="n">
-        <v>0.361</v>
+        <v>0.362</v>
       </c>
       <c r="W53" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="X53" t="n">
-        <v>96</v>
+        <v>95.8</v>
       </c>
       <c r="Y53" t="n">
         <v>246</v>
@@ -12953,10 +12953,10 @@
         </is>
       </c>
       <c r="V54" t="n">
-        <v>0.238</v>
+        <v>0.237</v>
       </c>
       <c r="W54" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="X54" t="n">
         <v>14.4</v>
@@ -13188,10 +13188,10 @@
         <v>0.029</v>
       </c>
       <c r="W55" t="n">
-        <v>7395</v>
+        <v>7412</v>
       </c>
       <c r="X55" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="Y55" t="n">
         <v>25</v>
@@ -13413,10 +13413,10 @@
         </is>
       </c>
       <c r="V56" t="n">
-        <v>0.84</v>
+        <v>0.841</v>
       </c>
       <c r="W56" t="n">
-        <v>3761</v>
+        <v>3758</v>
       </c>
       <c r="X56" t="n">
         <v>26.3</v>
@@ -13645,13 +13645,13 @@
         </is>
       </c>
       <c r="V57" t="n">
-        <v>0.232</v>
+        <v>0.231</v>
       </c>
       <c r="W57" t="n">
-        <v>1722</v>
+        <v>1727</v>
       </c>
       <c r="X57" t="n">
-        <v>18.2</v>
+        <v>18.3</v>
       </c>
       <c r="Y57" t="n">
         <v>-3</v>
@@ -13877,13 +13877,13 @@
         </is>
       </c>
       <c r="V58" t="n">
-        <v>0.247</v>
+        <v>0.246</v>
       </c>
       <c r="W58" t="n">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="X58" t="n">
-        <v>53</v>
+        <v>53.1</v>
       </c>
       <c r="Y58" t="n">
         <v>-4</v>
@@ -14109,13 +14109,13 @@
         </is>
       </c>
       <c r="V59" t="n">
-        <v>0.184</v>
+        <v>0.186</v>
       </c>
       <c r="W59" t="n">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="X59" t="n">
-        <v>15.7</v>
+        <v>15.5</v>
       </c>
       <c r="Y59" t="n">
         <v>-1</v>
@@ -14573,13 +14573,13 @@
         </is>
       </c>
       <c r="V61" t="n">
-        <v>0.264</v>
+        <v>0.263</v>
       </c>
       <c r="W61" t="n">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="X61" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="Y61" t="n">
         <v>-66</v>
@@ -14808,7 +14808,7 @@
         <v>0.04</v>
       </c>
       <c r="W62" t="n">
-        <v>3338</v>
+        <v>3335</v>
       </c>
       <c r="X62" t="n">
         <v>19.8</v>
@@ -15269,13 +15269,13 @@
         </is>
       </c>
       <c r="V64" t="n">
-        <v>0.106</v>
+        <v>0.105</v>
       </c>
       <c r="W64" t="n">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="X64" t="n">
-        <v>7.58</v>
+        <v>7.62</v>
       </c>
       <c r="Y64" t="n">
         <v>118</v>
@@ -15729,10 +15729,10 @@
         </is>
       </c>
       <c r="V66" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="W66" t="n">
-        <v>3885</v>
+        <v>3944</v>
       </c>
       <c r="X66" t="inlineStr"/>
       <c r="Y66" t="n">
@@ -15962,10 +15962,10 @@
         <v>0.076</v>
       </c>
       <c r="W67" t="n">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="X67" t="n">
-        <v>13.1</v>
+        <v>13</v>
       </c>
       <c r="Y67" t="n">
         <v>-8</v>
@@ -16194,7 +16194,7 @@
         <v>0</v>
       </c>
       <c r="W68" t="n">
-        <v>4937</v>
+        <v>4952</v>
       </c>
       <c r="X68" t="n">
         <v>11.6</v>
@@ -16658,10 +16658,10 @@
         <v>0.033</v>
       </c>
       <c r="W70" t="n">
-        <v>1472</v>
+        <v>1469</v>
       </c>
       <c r="X70" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="Y70" t="n">
         <v>11</v>
@@ -16890,7 +16890,7 @@
         <v>0</v>
       </c>
       <c r="W71" t="n">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="X71" t="n">
         <v>43.6</v>
@@ -17122,7 +17122,7 @@
         <v>0.003</v>
       </c>
       <c r="W72" t="n">
-        <v>12731</v>
+        <v>12734</v>
       </c>
       <c r="X72" t="n">
         <v>40.6</v>
@@ -17354,10 +17354,10 @@
         <v>0.031</v>
       </c>
       <c r="W73" t="n">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="X73" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="Y73" t="n">
         <v>27</v>
@@ -17586,7 +17586,7 @@
         <v>0.052</v>
       </c>
       <c r="W74" t="n">
-        <v>957</v>
+        <v>949</v>
       </c>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="n">
@@ -17816,10 +17816,10 @@
         <v>0</v>
       </c>
       <c r="W75" t="n">
-        <v>3812</v>
+        <v>3805</v>
       </c>
       <c r="X75" t="n">
-        <v>85.8</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="Y75" t="n">
         <v>42</v>
@@ -18048,10 +18048,10 @@
         <v>0.006</v>
       </c>
       <c r="W76" t="n">
-        <v>4828</v>
+        <v>4825</v>
       </c>
       <c r="X76" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="Y76" t="n">
         <v>23</v>
@@ -18276,7 +18276,7 @@
         <v>0</v>
       </c>
       <c r="W77" t="n">
-        <v>30214</v>
+        <v>30198</v>
       </c>
       <c r="X77" t="n">
         <v>226</v>
@@ -18508,10 +18508,10 @@
         <v>0</v>
       </c>
       <c r="W78" t="n">
-        <v>104998</v>
+        <v>105069</v>
       </c>
       <c r="X78" t="n">
-        <v>30.2</v>
+        <v>30.3</v>
       </c>
       <c r="Y78" t="n">
         <v>18</v>
@@ -18967,13 +18967,13 @@
         </is>
       </c>
       <c r="V80" t="n">
-        <v>0.234</v>
+        <v>0.231</v>
       </c>
       <c r="W80" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="X80" t="n">
-        <v>22.9</v>
+        <v>23.1</v>
       </c>
       <c r="Y80" t="n">
         <v>21</v>
@@ -19202,7 +19202,7 @@
         <v>0.026</v>
       </c>
       <c r="W81" t="n">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="X81" t="n">
         <v>37.3</v>
@@ -19419,10 +19419,10 @@
         </is>
       </c>
       <c r="V82" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="W82" t="n">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="X82" t="inlineStr"/>
       <c r="Y82" t="n">
@@ -20962,7 +20962,7 @@
         <v>-4</v>
       </c>
       <c r="F39" t="n">
-        <v>75</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="G39" t="n">
         <v>4.84</v>

</xml_diff>